<commit_message>
fix: normalise customer phone numbers to E.164
</commit_message>
<xml_diff>
--- a/data/customers.xlsx
+++ b/data/customers.xlsx
@@ -444,7 +444,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>+61400000001</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -459,7 +459,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>+61400000002</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -474,7 +474,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>+61400000003</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>+61400000004</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>+61400000005</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -519,7 +519,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>+61400000006</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>+61400000007</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -549,7 +549,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>+61400000008</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>+61400000009</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>+61400000010</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>+61400000011</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>+61400000012</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>+61400000013</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>+61400000014</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>+61400000015</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>+61400000016</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>+61400000017</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -699,7 +699,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>+61400000018</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>+61400000019</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>+61400000020</t>
+          <t>+19852391073</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: skip twilio signature validation in local dev
</commit_message>
<xml_diff>
--- a/data/customers.xlsx
+++ b/data/customers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shrey\.gemini\antigravity\outbound-assistant\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BABCCD55-86D9-4C35-9EFD-DC8640462E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E4ABAE-CCA3-43CC-95D9-9FA8CC3B2111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="24">
   <si>
     <t>customer_id</t>
   </si>
@@ -29,9 +29,6 @@
   </si>
   <si>
     <t>phone_number</t>
-  </si>
-  <si>
-    <t>+19852391073</t>
   </si>
   <si>
     <t>Olivia Bennett</t>
@@ -459,10 +456,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -470,10 +467,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s">
         <v>3</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -481,10 +478,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -492,10 +489,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" t="s">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -503,10 +500,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -514,10 +511,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" t="s">
-        <v>3</v>
+        <v>7</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -525,10 +522,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" t="s">
-        <v>3</v>
+        <v>8</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -536,10 +533,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" t="s">
-        <v>3</v>
+        <v>9</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -547,10 +544,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" t="s">
-        <v>3</v>
+        <v>10</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -558,10 +555,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" t="s">
-        <v>3</v>
+        <v>11</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -569,10 +566,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" t="s">
-        <v>3</v>
+        <v>12</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -580,10 +577,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" t="s">
-        <v>3</v>
+        <v>13</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -591,10 +588,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" t="s">
-        <v>3</v>
+        <v>14</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -602,10 +599,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" t="s">
-        <v>3</v>
+        <v>15</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -613,10 +610,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" t="s">
-        <v>3</v>
+        <v>16</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -624,10 +621,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" t="s">
-        <v>3</v>
+        <v>17</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -635,10 +632,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" t="s">
-        <v>3</v>
+        <v>18</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -646,10 +643,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" t="s">
-        <v>3</v>
+        <v>19</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -657,10 +654,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" t="s">
-        <v>3</v>
+        <v>20</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -668,10 +665,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" t="s">
-        <v>3</v>
+        <v>21</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>